<commit_message>
Update NBA player stats
</commit_message>
<xml_diff>
--- a/sportsref_download.xlsx
+++ b/sportsref_download.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ec4954651ec5d9f3/Documents/GitHub/nba-draft-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{5F1BC375-234C-4997-A88F-8507FDD67C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EE47672-F3A3-4CE3-BAE5-C0E3FD99FB00}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{5F1BC375-234C-4997-A88F-8507FDD67C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CB49932-9A46-4557-A2D4-C7D824489E80}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{B78C7215-33B7-4363-B67D-EB3EFE9C1878}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t>Rk</t>
   </si>
@@ -97,9 +97,6 @@
     <t>Donovan Mitchell</t>
   </si>
   <si>
-    <t>Cam Thomas</t>
-  </si>
-  <si>
     <t>Tyler Herro</t>
   </si>
   <si>
@@ -160,9 +157,6 @@
     <t>Darius Garland</t>
   </si>
   <si>
-    <t>Jordan Poole</t>
-  </si>
-  <si>
     <t>Coby White</t>
   </si>
   <si>
@@ -232,36 +226,21 @@
     <t>Immanuel Quickley</t>
   </si>
   <si>
-    <t>De'Andre Hunter</t>
-  </si>
-  <si>
     <t>Deni Avdija</t>
   </si>
   <si>
     <t>Keyonte George</t>
   </si>
   <si>
-    <t>Ivica Zubac</t>
-  </si>
-  <si>
     <t>Derrick White</t>
   </si>
   <si>
-    <t>Devin Vassell</t>
-  </si>
-  <si>
     <t>Paul George</t>
   </si>
   <si>
-    <t>Jalen Suggs</t>
-  </si>
-  <si>
     <t>Bennedict Mathurin</t>
   </si>
   <si>
-    <t>Kelly Oubre Jr.</t>
-  </si>
-  <si>
     <t>Chet Holmgren</t>
   </si>
   <si>
@@ -271,9 +250,6 @@
     <t>Aaron Gordon</t>
   </si>
   <si>
-    <t>P.J. Washington</t>
-  </si>
-  <si>
     <t>Josh Giddey</t>
   </si>
   <si>
@@ -298,9 +274,6 @@
     <t>Jabari Smith Jr.</t>
   </si>
   <si>
-    <t>Aaron Nesmith</t>
-  </si>
-  <si>
     <t>Jalen Duren</t>
   </si>
   <si>
@@ -335,6 +308,54 @@
   </si>
   <si>
     <t>VJ Edgecombe</t>
+  </si>
+  <si>
+    <t>Jayson Tatum</t>
+  </si>
+  <si>
+    <t>Ty Jerome</t>
+  </si>
+  <si>
+    <t>Saddiq Bey</t>
+  </si>
+  <si>
+    <t>Dejounte Murray</t>
+  </si>
+  <si>
+    <t>Matas Buzelis</t>
+  </si>
+  <si>
+    <t>Jarrett Allen</t>
+  </si>
+  <si>
+    <t>Russell Westbrook</t>
+  </si>
+  <si>
+    <t>Anthony Black</t>
+  </si>
+  <si>
+    <t>Ayo Dosunmu</t>
+  </si>
+  <si>
+    <t>Jaden McDaniels</t>
+  </si>
+  <si>
+    <t>Peyton Watson</t>
+  </si>
+  <si>
+    <t>Walker Kessler</t>
+  </si>
+  <si>
+    <t>Anfernee Simons</t>
+  </si>
+  <si>
+    <t>Kyrie Irving</t>
+  </si>
+  <si>
+    <t>Damian Lillard</t>
+  </si>
+  <si>
+    <t>Tyrese Haliburton</t>
   </si>
 </sst>
 </file>
@@ -1216,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{876D3B45-3B99-4C2A-A6C2-E5964AD0F784}">
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="3.73046875" bestFit="1" customWidth="1"/>
@@ -1235,7 +1256,7 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -1249,13 +1270,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2">
-        <v>33.700000000000003</v>
+        <v>33.5</v>
       </c>
       <c r="D2" s="2">
-        <v>8.5</v>
+        <v>7.7</v>
       </c>
       <c r="E2" s="2">
-        <v>8.6999999999999993</v>
+        <v>8.3000000000000007</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -1266,13 +1287,13 @@
         <v>4</v>
       </c>
       <c r="C3" s="2">
-        <v>32.1</v>
+        <v>31.1</v>
       </c>
       <c r="D3" s="2">
-        <v>4.9000000000000004</v>
+        <v>4.3</v>
       </c>
       <c r="E3" s="2">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -1280,16 +1301,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2">
-        <v>30.8</v>
+        <v>28.8</v>
       </c>
       <c r="D4" s="2">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2">
-        <v>7</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -1297,16 +1318,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2">
-        <v>30.7</v>
+        <v>28.7</v>
       </c>
       <c r="D5" s="2">
-        <v>4.5999999999999996</v>
+        <v>6.9</v>
       </c>
       <c r="E5" s="2">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -1314,16 +1335,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>29.8</v>
+        <v>28.3</v>
       </c>
       <c r="D6" s="2">
-        <v>12.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="E6" s="2">
-        <v>11</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -1331,16 +1352,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C7" s="2">
-        <v>29.4</v>
+        <v>27.9</v>
       </c>
       <c r="D7" s="2">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="E7" s="2">
-        <v>4.9000000000000004</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -1348,16 +1369,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C8" s="2">
-        <v>29.4</v>
+        <v>27.9</v>
       </c>
       <c r="D8" s="2">
-        <v>5.0999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="E8" s="2">
-        <v>3.8</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -1365,16 +1386,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C9" s="2">
-        <v>29.3</v>
+        <v>27.7</v>
       </c>
       <c r="D9" s="2">
-        <v>3.3</v>
+        <v>12.9</v>
       </c>
       <c r="E9" s="2">
-        <v>6.5</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -1385,13 +1406,13 @@
         <v>5</v>
       </c>
       <c r="C10" s="2">
-        <v>28.9</v>
+        <v>27.6</v>
       </c>
       <c r="D10" s="2">
-        <v>10.1</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="E10" s="2">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -1399,16 +1420,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C11" s="2">
-        <v>28.4</v>
+        <v>26.9</v>
       </c>
       <c r="D11" s="2">
-        <v>4.2</v>
+        <v>7.7</v>
       </c>
       <c r="E11" s="2">
-        <v>4.3</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -1416,16 +1437,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C12" s="2">
-        <v>27.8</v>
+        <v>26.7</v>
       </c>
       <c r="D12" s="2">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="E12" s="2">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -1433,16 +1454,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="C13" s="2">
         <v>26.6</v>
       </c>
       <c r="D13" s="2">
-        <v>5.2</v>
+        <v>3.6</v>
       </c>
       <c r="E13" s="2">
-        <v>6.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -1450,16 +1471,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C14" s="2">
-        <v>26.5</v>
+        <v>26.1</v>
       </c>
       <c r="D14" s="2">
-        <v>6.3</v>
+        <v>3.9</v>
       </c>
       <c r="E14" s="2">
-        <v>9.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -1467,16 +1488,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="C15" s="2">
-        <v>26.3</v>
+        <v>26</v>
       </c>
       <c r="D15" s="2">
-        <v>5</v>
+        <v>3.3</v>
       </c>
       <c r="E15" s="2">
-        <v>8</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -1484,16 +1505,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="C16" s="2">
-        <v>26.2</v>
+        <v>26</v>
       </c>
       <c r="D16" s="2">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="E16" s="2">
-        <v>3.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -1501,16 +1522,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="C17" s="2">
-        <v>25.7</v>
+        <v>25.4</v>
       </c>
       <c r="D17" s="2">
-        <v>7.3</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E17" s="2">
-        <v>3.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -1518,16 +1539,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="C18" s="2">
-        <v>25.6</v>
+        <v>25</v>
       </c>
       <c r="D18" s="2">
-        <v>7.1</v>
+        <v>11.5</v>
       </c>
       <c r="E18" s="2">
-        <v>6.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -1535,16 +1556,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="C19" s="2">
-        <v>25.6</v>
+        <v>24.2</v>
       </c>
       <c r="D19" s="2">
-        <v>4.3</v>
+        <v>6.9</v>
       </c>
       <c r="E19" s="2">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
@@ -1552,16 +1573,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="C20" s="2">
-        <v>25.4</v>
+        <v>24.2</v>
       </c>
       <c r="D20" s="2">
-        <v>4.3</v>
+        <v>7.1</v>
       </c>
       <c r="E20" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
@@ -1569,16 +1590,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="C21" s="2">
-        <v>25.2</v>
+        <v>24</v>
       </c>
       <c r="D21" s="2">
-        <v>5</v>
+        <v>6.6</v>
       </c>
       <c r="E21" s="2">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
@@ -1586,16 +1607,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="C22" s="2">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
       <c r="D22" s="2">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
       <c r="E22" s="2">
-        <v>6.8</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
@@ -1603,16 +1624,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="C23" s="2">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
       <c r="D23" s="2">
-        <v>10.4</v>
+        <v>4.8</v>
       </c>
       <c r="E23" s="2">
-        <v>8.3000000000000007</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
@@ -1620,16 +1641,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="C24" s="2">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
       <c r="D24" s="2">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="E24" s="2">
-        <v>2.7</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
@@ -1637,16 +1658,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="C25" s="2">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="D25" s="2">
-        <v>11.8</v>
+        <v>4.7</v>
       </c>
       <c r="E25" s="2">
-        <v>3.6</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
@@ -1654,16 +1675,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C26" s="2">
-        <v>23.2</v>
+        <v>22.5</v>
       </c>
       <c r="D26" s="2">
-        <v>5</v>
+        <v>10.3</v>
       </c>
       <c r="E26" s="2">
-        <v>2.2999999999999998</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
@@ -1671,16 +1692,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="C27" s="2">
-        <v>23.1</v>
+        <v>22.2</v>
       </c>
       <c r="D27" s="2">
-        <v>6.8</v>
+        <v>8.4</v>
       </c>
       <c r="E27" s="2">
-        <v>3.8</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
@@ -1688,16 +1709,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="C28" s="2">
-        <v>22.9</v>
+        <v>21.8</v>
       </c>
       <c r="D28" s="2">
-        <v>7.2</v>
+        <v>10</v>
       </c>
       <c r="E28" s="2">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
@@ -1705,16 +1726,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="C29" s="2">
-        <v>22.7</v>
+        <v>21.7</v>
       </c>
       <c r="D29" s="2">
-        <v>9.4</v>
+        <v>3.5</v>
       </c>
       <c r="E29" s="2">
-        <v>6.8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
@@ -1722,13 +1743,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C30" s="2">
-        <v>22.7</v>
+        <v>21.5</v>
       </c>
       <c r="D30" s="2">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="E30" s="2">
         <v>3.7</v>
@@ -1739,16 +1760,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C31" s="2">
-        <v>21.9</v>
+        <v>21.5</v>
       </c>
       <c r="D31" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="E31" s="2">
         <v>3.8</v>
-      </c>
-      <c r="E31" s="2">
-        <v>6.1</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
@@ -1756,16 +1777,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="C32" s="2">
-        <v>21.9</v>
+        <v>21.1</v>
       </c>
       <c r="D32" s="2">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
       <c r="E32" s="2">
-        <v>3.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
@@ -1773,16 +1794,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="C33" s="2">
-        <v>21.9</v>
+        <v>21</v>
       </c>
       <c r="D33" s="2">
-        <v>4.4000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="E33" s="2">
-        <v>2.4</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
@@ -1790,16 +1811,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C34" s="2">
-        <v>21.9</v>
+        <v>21</v>
       </c>
       <c r="D34" s="2">
-        <v>11.8</v>
+        <v>5.7</v>
       </c>
       <c r="E34" s="2">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
@@ -1807,16 +1828,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C35" s="2">
-        <v>21.8</v>
+        <v>20.9</v>
       </c>
       <c r="D35" s="2">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="E35" s="2">
-        <v>2.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.45">
@@ -1824,13 +1845,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="C36" s="2">
-        <v>21.7</v>
+        <v>20.8</v>
       </c>
       <c r="D36" s="2">
-        <v>5.9</v>
+        <v>3.4</v>
       </c>
       <c r="E36" s="2">
         <v>3.7</v>
@@ -1841,16 +1862,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="C37" s="2">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
       <c r="D37" s="2">
-        <v>3.1</v>
+        <v>4.3</v>
       </c>
       <c r="E37" s="2">
-        <v>1.7</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.45">
@@ -1858,16 +1879,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C38" s="2">
-        <v>21.4</v>
+        <v>20.6</v>
       </c>
       <c r="D38" s="2">
-        <v>1.4</v>
+        <v>5.2</v>
       </c>
       <c r="E38" s="2">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
@@ -1875,16 +1896,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="C39" s="2">
-        <v>20.8</v>
+        <v>20.5</v>
       </c>
       <c r="D39" s="2">
-        <v>3.5</v>
+        <v>4.8</v>
       </c>
       <c r="E39" s="2">
-        <v>5.0999999999999996</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
@@ -1895,10 +1916,10 @@
         <v>16</v>
       </c>
       <c r="C40" s="2">
-        <v>20.5</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="D40" s="2">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="E40" s="2">
         <v>2.8</v>
@@ -1909,16 +1930,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C41" s="2">
-        <v>20.5</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="D41" s="2">
-        <v>6.1</v>
+        <v>8.9</v>
       </c>
       <c r="E41" s="2">
-        <v>3.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.45">
@@ -1926,16 +1947,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="C42" s="2">
-        <v>20.399999999999999</v>
+        <v>20.2</v>
       </c>
       <c r="D42" s="2">
-        <v>6.3</v>
+        <v>3.6</v>
       </c>
       <c r="E42" s="2">
-        <v>3.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.45">
@@ -1943,16 +1964,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="C43" s="2">
-        <v>20.399999999999999</v>
+        <v>20.2</v>
       </c>
       <c r="D43" s="2">
-        <v>1.7</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="E43" s="2">
-        <v>8.8000000000000007</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.45">
@@ -1960,16 +1981,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>95</v>
+        <v>62</v>
       </c>
       <c r="C44" s="2">
-        <v>20.2</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="D44" s="2">
-        <v>3.5</v>
+        <v>10</v>
       </c>
       <c r="E44" s="2">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
@@ -1977,16 +1998,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C45" s="2">
-        <v>20.2</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="D45" s="2">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="E45" s="2">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
@@ -1994,16 +2015,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C46" s="2">
-        <v>20.2</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="D46" s="2">
-        <v>3</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="E46" s="2">
-        <v>2.2999999999999998</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.45">
@@ -2011,16 +2032,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C47" s="2">
         <v>20.100000000000001</v>
       </c>
       <c r="D47" s="2">
-        <v>8.3000000000000007</v>
+        <v>11.9</v>
       </c>
       <c r="E47" s="2">
-        <v>4.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.45">
@@ -2028,16 +2049,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="C48" s="2">
         <v>20</v>
       </c>
       <c r="D48" s="2">
-        <v>4</v>
+        <v>5.6</v>
       </c>
       <c r="E48" s="2">
-        <v>2.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.45">
@@ -2045,16 +2066,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C49" s="2">
-        <v>20</v>
+        <v>19.7</v>
       </c>
       <c r="D49" s="2">
-        <v>5.2</v>
+        <v>2.8</v>
       </c>
       <c r="E49" s="2">
-        <v>7.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.45">
@@ -2065,13 +2086,13 @@
         <v>84</v>
       </c>
       <c r="C50" s="2">
-        <v>19.8</v>
+        <v>19.5</v>
       </c>
       <c r="D50" s="2">
-        <v>9.1999999999999993</v>
+        <v>10.5</v>
       </c>
       <c r="E50" s="2">
-        <v>9.1999999999999993</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.45">
@@ -2079,16 +2100,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C51" s="2">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="D51" s="2">
-        <v>5.4</v>
+        <v>3.3</v>
       </c>
       <c r="E51" s="2">
-        <v>8.5</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.45">
@@ -2096,16 +2117,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="C52" s="2">
-        <v>19.7</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="D52" s="2">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="E52" s="2">
-        <v>4.9000000000000004</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.45">
@@ -2113,16 +2134,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C53" s="2">
-        <v>19.399999999999999</v>
+        <v>19.3</v>
       </c>
       <c r="D53" s="2">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="E53" s="2">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.45">
@@ -2130,16 +2151,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="C54" s="2">
-        <v>19.399999999999999</v>
+        <v>19.2</v>
       </c>
       <c r="D54" s="2">
-        <v>6.4</v>
+        <v>2.8</v>
       </c>
       <c r="E54" s="2">
-        <v>3.8</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.45">
@@ -2147,16 +2168,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>98</v>
+        <v>44</v>
       </c>
       <c r="C55" s="2">
-        <v>19.3</v>
+        <v>18.8</v>
       </c>
       <c r="D55" s="2">
-        <v>5.0999999999999996</v>
+        <v>2.4</v>
       </c>
       <c r="E55" s="2">
-        <v>3.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.45">
@@ -2164,16 +2185,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="C56" s="2">
-        <v>19.2</v>
+        <v>18.7</v>
       </c>
       <c r="D56" s="2">
-        <v>7.9</v>
+        <v>3.3</v>
       </c>
       <c r="E56" s="2">
-        <v>5.0999999999999996</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.45">
@@ -2181,16 +2202,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="C57" s="2">
-        <v>19.2</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="D57" s="2">
-        <v>5.6</v>
+        <v>3.8</v>
       </c>
       <c r="E57" s="2">
-        <v>3.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.45">
@@ -2198,16 +2219,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="C58" s="2">
-        <v>19</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="D58" s="2">
-        <v>4.5999999999999996</v>
+        <v>3.5</v>
       </c>
       <c r="E58" s="2">
-        <v>4.5</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.45">
@@ -2215,16 +2236,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="C59" s="2">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="D59" s="2">
-        <v>3.3</v>
+        <v>5.3</v>
       </c>
       <c r="E59" s="2">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.45">
@@ -2232,13 +2253,13 @@
         <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="C60" s="2">
-        <v>18.899999999999999</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="D60" s="2">
-        <v>9.3000000000000007</v>
+        <v>2.9</v>
       </c>
       <c r="E60" s="2">
         <v>4.0999999999999996</v>
@@ -2249,16 +2270,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C61" s="2">
-        <v>18.8</v>
+        <v>18.3</v>
       </c>
       <c r="D61" s="2">
-        <v>5.9</v>
+        <v>7.8</v>
       </c>
       <c r="E61" s="2">
-        <v>1.3</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.45">
@@ -2266,13 +2287,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="C62" s="2">
-        <v>18.7</v>
+        <v>18.2</v>
       </c>
       <c r="D62" s="2">
-        <v>3.4</v>
+        <v>9</v>
       </c>
       <c r="E62" s="2">
         <v>3.6</v>
@@ -2283,16 +2304,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="C63" s="2">
-        <v>18.600000000000001</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="D63" s="2">
-        <v>5.2</v>
+        <v>7.5</v>
       </c>
       <c r="E63" s="2">
-        <v>7</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.45">
@@ -2300,16 +2321,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="C64" s="2">
-        <v>18.3</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="D64" s="2">
-        <v>10.8</v>
+        <v>2</v>
       </c>
       <c r="E64" s="2">
-        <v>1.8</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.45">
@@ -2317,16 +2338,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="C65" s="2">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="D65" s="2">
-        <v>4.2</v>
+        <v>3.6</v>
       </c>
       <c r="E65" s="2">
-        <v>5.0999999999999996</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.45">
@@ -2334,16 +2355,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="C66" s="2">
-        <v>18.2</v>
+        <v>17.7</v>
       </c>
       <c r="D66" s="2">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="E66" s="2">
-        <v>2.2000000000000002</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.45">
@@ -2351,16 +2372,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C67" s="2">
-        <v>18.2</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="D67" s="2">
-        <v>8.3000000000000007</v>
+        <v>5.4</v>
       </c>
       <c r="E67" s="2">
-        <v>3</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.45">
@@ -2368,16 +2389,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C68" s="2">
-        <v>18</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="D68" s="2">
-        <v>9.5</v>
+        <v>3.4</v>
       </c>
       <c r="E68" s="2">
-        <v>2.4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.45">
@@ -2385,16 +2406,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="C69" s="2">
-        <v>18</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="D69" s="2">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="E69" s="2">
-        <v>2</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.45">
@@ -2402,16 +2423,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C70" s="2">
-        <v>17.899999999999999</v>
+        <v>17.3</v>
       </c>
       <c r="D70" s="2">
-        <v>7.8</v>
+        <v>5.3</v>
       </c>
       <c r="E70" s="2">
-        <v>1.6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.45">
@@ -2419,16 +2440,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>44</v>
+        <v>91</v>
       </c>
       <c r="C71" s="2">
-        <v>17.899999999999999</v>
+        <v>17.3</v>
       </c>
       <c r="D71" s="2">
-        <v>3.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="E71" s="2">
-        <v>3.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.45">
@@ -2436,16 +2457,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="C72" s="2">
-        <v>17.899999999999999</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="D72" s="2">
-        <v>7.3</v>
+        <v>5.8</v>
       </c>
       <c r="E72" s="2">
-        <v>5.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.45">
@@ -2453,16 +2474,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="C73" s="2">
-        <v>17.7</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="D73" s="2">
-        <v>3.5</v>
+        <v>8.9</v>
       </c>
       <c r="E73" s="2">
-        <v>7.7</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.45">
@@ -2470,16 +2491,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C74" s="2">
-        <v>17.600000000000001</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="D74" s="2">
-        <v>5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="E74" s="2">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.45">
@@ -2487,16 +2508,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="C75" s="2">
-        <v>17.399999999999999</v>
+        <v>17</v>
       </c>
       <c r="D75" s="2">
-        <v>2.2999999999999998</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="E75" s="2">
-        <v>6.5</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.45">
@@ -2504,16 +2525,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="C76" s="2">
-        <v>17.3</v>
+        <v>17</v>
       </c>
       <c r="D76" s="2">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
       <c r="E76" s="2">
-        <v>7.1</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.45">
@@ -2521,16 +2542,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="C77" s="2">
-        <v>17.2</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="D77" s="2">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="E77" s="2">
-        <v>3.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.45">
@@ -2538,16 +2559,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="C78" s="2">
-        <v>17.2</v>
+        <v>16.7</v>
       </c>
       <c r="D78" s="2">
-        <v>4.5</v>
+        <v>5.2</v>
       </c>
       <c r="E78" s="2">
-        <v>5.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.45">
@@ -2555,16 +2576,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C79" s="2">
-        <v>17.2</v>
+        <v>16.7</v>
       </c>
       <c r="D79" s="2">
-        <v>12.3</v>
+        <v>5.2</v>
       </c>
       <c r="E79" s="2">
-        <v>3.7</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.45">
@@ -2572,16 +2593,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="C80" s="2">
-        <v>17.100000000000001</v>
+        <v>16.7</v>
       </c>
       <c r="D80" s="2">
-        <v>4.0999999999999996</v>
+        <v>5.3</v>
       </c>
       <c r="E80" s="2">
-        <v>5.8</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.45">
@@ -2589,16 +2610,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="C81" s="2">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
       <c r="D81" s="2">
-        <v>4.5999999999999996</v>
+        <v>5.4</v>
       </c>
       <c r="E81" s="2">
-        <v>4.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.45">
@@ -2606,16 +2627,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="C82" s="2">
-        <v>16.8</v>
+        <v>16.5</v>
       </c>
       <c r="D82" s="2">
-        <v>5.0999999999999996</v>
+        <v>3</v>
       </c>
       <c r="E82" s="2">
-        <v>1.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.45">
@@ -2623,16 +2644,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="C83" s="2">
-        <v>16.7</v>
+        <v>16.5</v>
       </c>
       <c r="D83" s="2">
-        <v>5.3</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E83" s="2">
-        <v>8.3000000000000007</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.45">
@@ -2640,16 +2661,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="C84" s="2">
-        <v>16.3</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="D84" s="2">
-        <v>2.7</v>
+        <v>4</v>
       </c>
       <c r="E84" s="2">
-        <v>4.0999999999999996</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.45">
@@ -2657,16 +2678,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="C85" s="2">
         <v>16.3</v>
       </c>
       <c r="D85" s="2">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="E85" s="2">
-        <v>3.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.45">
@@ -2674,16 +2695,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="C86" s="2">
-        <v>16.100000000000001</v>
+        <v>16.3</v>
       </c>
       <c r="D86" s="2">
-        <v>4.3</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="E86" s="2">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.45">
@@ -2691,16 +2712,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="C87" s="2">
-        <v>15.9</v>
+        <v>16.3</v>
       </c>
       <c r="D87" s="2">
-        <v>5.5</v>
+        <v>7.4</v>
       </c>
       <c r="E87" s="2">
-        <v>4.5999999999999996</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.45">
@@ -2708,16 +2729,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C88" s="2">
-        <v>15.9</v>
+        <v>16.2</v>
       </c>
       <c r="D88" s="2">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="E88" s="2">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.45">
@@ -2725,16 +2746,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="C89" s="2">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="D89" s="2">
         <v>5.6</v>
       </c>
       <c r="E89" s="2">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.45">
@@ -2742,16 +2763,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C90" s="2">
         <v>15.8</v>
       </c>
       <c r="D90" s="2">
-        <v>9.1</v>
+        <v>11.4</v>
       </c>
       <c r="E90" s="2">
-        <v>3.4</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.45">
@@ -2759,13 +2780,13 @@
         <v>90</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C91" s="2">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="D91" s="2">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="E91" s="2">
         <v>1.9</v>
@@ -2776,16 +2797,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="C92" s="2">
-        <v>15.6</v>
+        <v>15.4</v>
       </c>
       <c r="D92" s="2">
-        <v>7.4</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E92" s="2">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.45">
@@ -2793,16 +2814,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="C93" s="2">
-        <v>15.6</v>
+        <v>15.4</v>
       </c>
       <c r="D93" s="2">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="E93" s="2">
-        <v>2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.45">
@@ -2810,16 +2831,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="C94" s="2">
-        <v>15.6</v>
+        <v>15.4</v>
       </c>
       <c r="D94" s="2">
-        <v>11.1</v>
+        <v>5</v>
       </c>
       <c r="E94" s="2">
-        <v>2.5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.45">
@@ -2827,16 +2848,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="C95" s="2">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="D95" s="2">
-        <v>2</v>
+        <v>4.8</v>
       </c>
       <c r="E95" s="2">
-        <v>2</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.45">
@@ -2844,16 +2865,16 @@
         <v>95</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="C96" s="2">
-        <v>15.5</v>
+        <v>15.2</v>
       </c>
       <c r="D96" s="2">
-        <v>4.5</v>
+        <v>7.6</v>
       </c>
       <c r="E96" s="2">
-        <v>1.5</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.45">
@@ -2861,16 +2882,16 @@
         <v>96</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C97" s="2">
-        <v>15.4</v>
+        <v>15.2</v>
       </c>
       <c r="D97" s="2">
-        <v>3.7</v>
+        <v>5.4</v>
       </c>
       <c r="E97" s="2">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.45">
@@ -2878,16 +2899,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="C98" s="2">
-        <v>15.4</v>
+        <v>15.1</v>
       </c>
       <c r="D98" s="2">
-        <v>4.0999999999999996</v>
+        <v>8.4</v>
       </c>
       <c r="E98" s="2">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.45">
@@ -2895,16 +2916,16 @@
         <v>98</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="C99" s="2">
-        <v>15.3</v>
+        <v>15</v>
       </c>
       <c r="D99" s="2">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="E99" s="2">
-        <v>2.1</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.45">
@@ -2912,16 +2933,16 @@
         <v>99</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="C100" s="2">
-        <v>15.3</v>
+        <v>14.8</v>
       </c>
       <c r="D100" s="2">
-        <v>2.1</v>
+        <v>3.4</v>
       </c>
       <c r="E100" s="2">
-        <v>4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.45">
@@ -2929,16 +2950,135 @@
         <v>100</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>66</v>
+        <v>105</v>
       </c>
       <c r="C101" s="2">
-        <v>15.2</v>
+        <v>14.8</v>
       </c>
       <c r="D101" s="2">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="E101" s="2">
-        <v>2</v>
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A102" s="1">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C102" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="D102" s="2">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="E102" s="2">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A103" s="1">
+        <v>102</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C103" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="D103" s="2">
+        <v>3.8</v>
+      </c>
+      <c r="E103" s="2">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A104" s="1">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C104" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="D104" s="2">
+        <v>10.8</v>
+      </c>
+      <c r="E104" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A105" s="1">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C105" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="D105" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="E105" s="2">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A106" s="1">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C106" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="D106" s="2">
+        <v>4.8</v>
+      </c>
+      <c r="E106" s="2">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A107" s="1">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C107" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="D107" s="2">
+        <v>4.7</v>
+      </c>
+      <c r="E107" s="2">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A108" s="1">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C108" s="2">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="D108" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="E108" s="2">
+        <v>9.1999999999999993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>